<commit_message>
Changes TARGCENT to TCENT`n` which quantifies the fraction of a observation where data was within 10,20,30 pixels from center.
</commit_message>
<xml_diff>
--- a/src/pandorafits/formats/nirda/level2_nirda.xlsx
+++ b/src/pandorafits/formats/nirda/level2_nirda.xlsx
@@ -745,7 +745,6 @@
           <t>NAXIS1</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>32</t>
@@ -763,7 +762,6 @@
           <t>NAXIS2</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>250</t>
@@ -781,7 +779,6 @@
           <t>PCOUNT</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>0</t>
@@ -799,7 +796,6 @@
           <t>GCOUNT</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
           <t>1</t>
@@ -849,7 +845,6 @@
           <t>row</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -867,7 +862,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -875,13 +869,11 @@
           <t>TUNIT1</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
           <t>pix</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -899,7 +891,6 @@
           <t>drow</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -917,7 +908,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -925,13 +915,11 @@
           <t>TUNIT2</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
           <t>pix</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -949,7 +937,6 @@
           <t>wavelength</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -967,7 +954,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -975,13 +961,11 @@
           <t>TUNIT3</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
           <t>um</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -999,7 +983,6 @@
           <t>sensitivity</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1017,7 +1000,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1025,13 +1007,11 @@
           <t>TUNIT4</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
           <t>cm2 Angstrom count erg-1</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1049,7 +1029,6 @@
           <t>WAVELENGTH_SOLUTION</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1057,7 +1036,6 @@
           <t>CHECKSUM</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
           <t>9M5MFM5K9M5KEM5K</t>
@@ -1075,7 +1053,6 @@
           <t>DATASUM</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
           <t>2322579671</t>
@@ -1195,7 +1172,6 @@
           <t>NAXIS1</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>80</t>
@@ -1213,7 +1189,6 @@
           <t>NAXIS2</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>250</t>
@@ -1231,7 +1206,6 @@
           <t>PCOUNT</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>0</t>
@@ -1249,7 +1223,6 @@
           <t>GCOUNT</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
           <t>1</t>
@@ -1289,7 +1262,6 @@
           <t>CONTAM</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
           <t>1.45948781805724e-05</t>
@@ -1307,7 +1279,6 @@
           <t>COMPLTE</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
           <t>1.0001196545262074</t>
@@ -1325,7 +1296,6 @@
           <t>TOTAP</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
           <t>6054546.661906874</t>
@@ -1343,13 +1313,11 @@
           <t>RA</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
           <t>307.85996711980397</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1357,13 +1325,11 @@
           <t>DEC</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
           <t>39.93898084328189</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1371,13 +1337,11 @@
           <t>ROW</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
           <t>1086.4587761921186</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1385,13 +1349,11 @@
           <t>COLUMN</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr">
         <is>
           <t>1775.530593149113</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1399,13 +1361,11 @@
           <t>GAIA_ID</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr">
         <is>
           <t>2064327278651198336</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1413,7 +1373,6 @@
           <t>IMSIZE0</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
           <t>250</t>
@@ -1431,7 +1390,6 @@
           <t>IMCRNR0</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
           <t>962</t>
@@ -1449,7 +1407,6 @@
           <t>IMSIZE1</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
           <t>80</t>
@@ -1467,7 +1424,6 @@
           <t>IMCRNR1</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
           <t>1737</t>
@@ -1485,7 +1441,6 @@
           <t>CHECKSUM</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
           <t>eD6kf93ieC3ie93i</t>
@@ -1503,7 +1458,6 @@
           <t>DATASUM</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
           <t>178391814</t>
@@ -1623,7 +1577,6 @@
           <t>NAXIS1</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>80</t>
@@ -1641,7 +1594,6 @@
           <t>NAXIS2</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>250</t>
@@ -1659,7 +1611,6 @@
           <t>PCOUNT</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>0</t>
@@ -1677,7 +1628,6 @@
           <t>GCOUNT</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
           <t>1</t>
@@ -1695,7 +1645,6 @@
           <t>WCSAXES</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
           <t>2</t>
@@ -1713,7 +1662,6 @@
           <t>CRPIX1</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
           <t>44.0</t>
@@ -1731,7 +1679,6 @@
           <t>CRPIX2</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
           <t>123.0</t>
@@ -1749,7 +1696,6 @@
           <t>PC1_1</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
           <t>0.92523789004974</t>
@@ -1767,7 +1713,6 @@
           <t>PC1_2</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
           <t>-0.3793874626504</t>
@@ -1785,7 +1730,6 @@
           <t>PC2_1</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
           <t>0.3793874626504</t>
@@ -1803,7 +1747,6 @@
           <t>PC2_2</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
           <t>0.92523789004974</t>
@@ -1821,7 +1764,6 @@
           <t>CDELT1</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr">
         <is>
           <t>0.00033055555555556</t>
@@ -1839,7 +1781,6 @@
           <t>CDELT2</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr">
         <is>
           <t>0.00033055555555556</t>
@@ -1857,7 +1798,6 @@
           <t>CUNIT1</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
           <t>deg</t>
@@ -1875,7 +1815,6 @@
           <t>CUNIT2</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
           <t>deg</t>
@@ -1893,7 +1832,6 @@
           <t>CTYPE1</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
           <t>RA---TAN</t>
@@ -1911,7 +1849,6 @@
           <t>CTYPE2</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
           <t>DEC--TAN</t>
@@ -1929,7 +1866,6 @@
           <t>CRVAL1</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
           <t>307.86215209961</t>
@@ -1947,7 +1883,6 @@
           <t>CRVAL2</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
           <t>39.938789367676</t>
@@ -1965,7 +1900,6 @@
           <t>LONPOLE</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
           <t>180.0</t>
@@ -1983,7 +1917,6 @@
           <t>LATPOLE</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
           <t>39.938789367676</t>
@@ -2001,7 +1934,6 @@
           <t>MJDREF</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
           <t>0.0</t>
@@ -2019,7 +1951,6 @@
           <t>RADESYS</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
           <t>ICRS</t>
@@ -2059,7 +1990,6 @@
           <t>IMSIZE0</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
           <t>250</t>
@@ -2077,7 +2007,6 @@
           <t>IMCRNR0</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
           <t>962</t>
@@ -2095,7 +2024,6 @@
           <t>IMSIZE1</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
           <t>80</t>
@@ -2113,7 +2041,6 @@
           <t>IMCRNR1</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
           <t>1737</t>
@@ -2131,7 +2058,6 @@
           <t>CHECKSUM</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
           <t>LF7VOD4VLD4VLD4V</t>
@@ -2149,7 +2075,6 @@
           <t>DATASUM</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
           <t>4243662291</t>
@@ -2269,7 +2194,6 @@
           <t>NAXIS1</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>250</t>
@@ -2287,7 +2211,6 @@
           <t>NAXIS2</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>387</t>
@@ -2305,7 +2228,6 @@
           <t>PCOUNT</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>0</t>
@@ -2323,7 +2245,6 @@
           <t>GCOUNT</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
           <t>1</t>
@@ -2341,13 +2262,11 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
           <t>ct / s</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2377,7 +2296,6 @@
           <t>CHECKSUM</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
           <t>a0AUc06Ta0ATa03T</t>
@@ -2395,7 +2313,6 @@
           <t>DATASUM</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
           <t>4262218308</t>
@@ -2418,7 +2335,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D108"/>
+  <dimension ref="A1:D110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2525,7 +2442,6 @@
           <t>True</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2555,7 +2471,6 @@
           <t>NEXTEND</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>2</t>
@@ -2573,7 +2488,6 @@
           <t>SIMDATA</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
           <t>False</t>
@@ -2591,7 +2505,6 @@
           <t>SCIDATA</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
           <t>True</t>
@@ -2675,7 +2588,6 @@
           <t>CREATOR</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
           <t>Pandora MOC</t>
@@ -2693,7 +2605,6 @@
           <t>CRSOFTV</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
           <t>v3.06</t>
@@ -2711,7 +2622,6 @@
           <t>COMPTYPE</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
           <t>1</t>
@@ -2729,7 +2639,6 @@
           <t>TRANSID</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr">
         <is>
           <t>0</t>
@@ -2747,7 +2656,6 @@
           <t>TARG_ID</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr">
         <is>
           <t>KELT-9b</t>
@@ -2765,7 +2673,6 @@
           <t>FILENAME</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
           <t>/sssp/data/2026/08/15/2026-08-15__06-44-18_InfImg_KELT-9b_d0080x0250x3096_b1_e01_i387_g02_d16_r04.sp</t>
@@ -2783,7 +2690,6 @@
           <t>BINSIZE</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
           <t>1</t>
@@ -2801,7 +2707,6 @@
           <t>BITDEPTH</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
           <t>32</t>
@@ -2819,7 +2724,6 @@
           <t>BITSPIX</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
           <t>16</t>
@@ -2837,7 +2741,6 @@
           <t>ROISTRTX</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
           <t>1737</t>
@@ -2855,7 +2758,6 @@
           <t>ROISTRTY</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
           <t>962</t>
@@ -2873,7 +2775,6 @@
           <t>ROISTRTZ</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
           <t>0</t>
@@ -2891,7 +2792,6 @@
           <t>ROISIZEX</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
           <t>80</t>
@@ -2909,7 +2809,6 @@
           <t>ROISIZEY</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
           <t>250</t>
@@ -2927,7 +2826,6 @@
           <t>ROISIZEZ</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
           <t>774</t>
@@ -2945,7 +2843,6 @@
           <t>RICEX</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
           <t>5</t>
@@ -2963,7 +2860,6 @@
           <t>RICEY</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
           <t>28</t>
@@ -2981,7 +2877,6 @@
           <t>CORSTIME</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
           <t>840091495</t>
@@ -2999,7 +2894,6 @@
           <t>FINETIME</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
           <t>832000000</t>
@@ -3017,7 +2911,6 @@
           <t>COMMAND</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
           <t>10</t>
@@ -3035,7 +2928,6 @@
           <t>CONFIG1</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
           <t>53251</t>
@@ -3053,7 +2945,6 @@
           <t>CONFIG2</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
           <t>0</t>
@@ -3071,7 +2962,6 @@
           <t>CONFIG3</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
           <t>0</t>
@@ -3089,7 +2979,6 @@
           <t>GAINREG</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
           <t>37002</t>
@@ -3107,7 +2996,6 @@
           <t>RESETS1</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
           <t>259</t>
@@ -3125,7 +3013,6 @@
           <t>RESETS2</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
           <t>1</t>
@@ -3143,7 +3030,6 @@
           <t>DROPS1</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
           <t>1</t>
@@ -3161,7 +3047,6 @@
           <t>DROPS2</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
           <t>16</t>
@@ -3179,7 +3064,6 @@
           <t>DROPS3</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
           <t>0</t>
@@ -3197,7 +3081,6 @@
           <t>READS</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
           <t>4</t>
@@ -3215,7 +3098,6 @@
           <t>GRPS</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
           <t>2</t>
@@ -3233,7 +3115,6 @@
           <t>INTEGRTS</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
           <t>387</t>
@@ -3251,7 +3132,6 @@
           <t>EXPOSRES</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
           <t>1</t>
@@ -3269,7 +3149,6 @@
           <t>ENDDELAY</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
           <t>0</t>
@@ -3287,7 +3166,6 @@
           <t>RSTSINC</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
           <t>0</t>
@@ -3305,7 +3183,6 @@
           <t>DRPSINC</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr">
         <is>
           <t>0</t>
@@ -3323,7 +3200,6 @@
           <t>FRMSTOT</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr">
         <is>
           <t>10320</t>
@@ -3341,7 +3217,6 @@
           <t>FRMSEXP</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr">
         <is>
           <t>3096</t>
@@ -3359,7 +3234,6 @@
           <t>FRMSACQ</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr">
         <is>
           <t>3096</t>
@@ -3377,7 +3251,6 @@
           <t>GRPSAVGD</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr">
         <is>
           <t>1</t>
@@ -3395,7 +3268,6 @@
           <t>PAMPGAIN</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr">
         <is>
           <t>5.65685</t>
@@ -3413,7 +3285,6 @@
           <t>FRMTIME</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr">
         <is>
           <t>231</t>
@@ -3431,7 +3302,6 @@
           <t>TSIDECAR</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr">
         <is>
           <t>3.3816466331481934</t>
@@ -3449,7 +3319,6 @@
           <t>TCOMPRJT</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr">
         <is>
           <t>278.990966796875</t>
@@ -3467,7 +3336,6 @@
           <t>TCLDTIP1</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr"/>
       <c r="C57" t="inlineStr">
         <is>
           <t>131.50372314453125</t>
@@ -3485,7 +3353,6 @@
           <t>TCLDTIP2</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr"/>
       <c r="C58" t="inlineStr">
         <is>
           <t>120.03438568115234</t>
@@ -3503,7 +3370,6 @@
           <t>CHECKSUM</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr">
         <is>
           <t>9agDGWgC9agCEWgC</t>
@@ -3521,7 +3387,6 @@
           <t>DATASUM</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr">
         <is>
           <t>0</t>
@@ -3539,13 +3404,11 @@
           <t>FIXED</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr"/>
       <c r="C61" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3553,13 +3416,11 @@
           <t>PFSOFTV</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr"/>
       <c r="C62" t="inlineStr">
         <is>
           <t>0.6.0</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3567,13 +3428,11 @@
           <t>PRSOFTV</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr"/>
       <c r="C63" t="inlineStr">
         <is>
           <t>2.9.1</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3581,13 +3440,11 @@
           <t>PFCLASS</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr"/>
       <c r="C64" t="inlineStr">
         <is>
           <t>NIRDALevel2HDUList</t>
         </is>
       </c>
-      <c r="D64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3595,7 +3452,6 @@
           <t>PFTIME</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr"/>
       <c r="C65" t="inlineStr">
         <is>
           <t>2026-09-09T19:46:08.484</t>
@@ -3613,7 +3469,6 @@
           <t>TARG_RA</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr"/>
       <c r="C66" t="inlineStr">
         <is>
           <t>307.8599548339844</t>
@@ -3631,7 +3486,6 @@
           <t>TARG_DEC</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr"/>
       <c r="C67" t="inlineStr">
         <is>
           <t>39.9389762878418</t>
@@ -3649,7 +3503,6 @@
           <t>RA</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr"/>
       <c r="C68" t="inlineStr">
         <is>
           <t>307.86216741569376</t>
@@ -3667,7 +3520,6 @@
           <t>DEC</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr"/>
       <c r="C69" t="inlineStr">
         <is>
           <t>39.93878532835476</t>
@@ -3685,7 +3537,6 @@
           <t>ROLL</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr"/>
       <c r="C70" t="inlineStr">
         <is>
           <t>247.7078167885557</t>
@@ -3703,7 +3554,6 @@
           <t>POSX</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr"/>
       <c r="C71" t="inlineStr">
         <is>
           <t>1775.498998065344</t>
@@ -3721,7 +3571,6 @@
           <t>POSY</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr"/>
       <c r="C72" t="inlineStr">
         <is>
           <t>1086.4568375724239</t>
@@ -3739,7 +3588,6 @@
           <t>GAIADR3</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr"/>
       <c r="C73" t="inlineStr">
         <is>
           <t>Gaia DR3 2064327278651198336</t>
@@ -3757,7 +3605,6 @@
           <t>GAIARA</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr"/>
       <c r="C74" t="inlineStr">
         <is>
           <t>307.8599027970418</t>
@@ -3775,7 +3622,6 @@
           <t>GAIADEC</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr"/>
       <c r="C75" t="inlineStr">
         <is>
           <t>39.93891900336815</t>
@@ -3793,7 +3639,6 @@
           <t>PARALLAX</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr"/>
       <c r="C76" t="inlineStr">
         <is>
           <t>4.825836101438949</t>
@@ -3811,7 +3656,6 @@
           <t>PMRA</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr"/>
       <c r="C77" t="inlineStr">
         <is>
           <t>16.716578051403854</t>
@@ -3829,7 +3673,6 @@
           <t>PMDEC</t>
         </is>
       </c>
-      <c r="B78" t="inlineStr"/>
       <c r="C78" t="inlineStr">
         <is>
           <t>20.96090596020299</t>
@@ -3847,7 +3690,6 @@
           <t>2MASSID</t>
         </is>
       </c>
-      <c r="B79" t="inlineStr"/>
       <c r="C79" t="inlineStr">
         <is>
           <t>2MASS J20312634+3956196</t>
@@ -3865,7 +3707,6 @@
           <t>J_M</t>
         </is>
       </c>
-      <c r="B80" t="inlineStr"/>
       <c r="C80" t="inlineStr">
         <is>
           <t>7.458</t>
@@ -3883,7 +3724,6 @@
           <t>H_M</t>
         </is>
       </c>
-      <c r="B81" t="inlineStr"/>
       <c r="C81" t="inlineStr">
         <is>
           <t>7.492</t>
@@ -3901,7 +3741,6 @@
           <t>K_M</t>
         </is>
       </c>
-      <c r="B82" t="inlineStr"/>
       <c r="C82" t="inlineStr">
         <is>
           <t>7.482</t>
@@ -3919,7 +3758,6 @@
           <t>G_M</t>
         </is>
       </c>
-      <c r="B83" t="inlineStr"/>
       <c r="C83" t="inlineStr">
         <is>
           <t>7.5902658552584015</t>
@@ -3937,7 +3775,6 @@
           <t>BP_M</t>
         </is>
       </c>
-      <c r="B84" t="inlineStr"/>
       <c r="C84" t="inlineStr">
         <is>
           <t>7.594925828938212</t>
@@ -3955,7 +3792,6 @@
           <t>RP_M</t>
         </is>
       </c>
-      <c r="B85" t="inlineStr"/>
       <c r="C85" t="inlineStr">
         <is>
           <t>7.552309075270038</t>
@@ -3973,7 +3809,6 @@
           <t>TEFF</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr"/>
       <c r="C86" t="inlineStr">
         <is>
           <t>9951.392</t>
@@ -3991,7 +3826,6 @@
           <t>LOGG</t>
         </is>
       </c>
-      <c r="B87" t="inlineStr"/>
       <c r="C87" t="inlineStr">
         <is>
           <t>3.9497</t>
@@ -4009,13 +3843,11 @@
           <t>COLLAPS</t>
         </is>
       </c>
-      <c r="B88" t="inlineStr"/>
       <c r="C88" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -4023,7 +3855,6 @@
           <t>BKG10</t>
         </is>
       </c>
-      <c r="B89" t="inlineStr"/>
       <c r="C89" t="inlineStr">
         <is>
           <t>119.15584415584416</t>
@@ -4041,7 +3872,6 @@
           <t>BKG50</t>
         </is>
       </c>
-      <c r="B90" t="inlineStr"/>
       <c r="C90" t="inlineStr">
         <is>
           <t>157.034632034632</t>
@@ -4059,7 +3889,6 @@
           <t>BKG90</t>
         </is>
       </c>
-      <c r="B91" t="inlineStr"/>
       <c r="C91" t="inlineStr">
         <is>
           <t>188.3116883116883</t>
@@ -4077,7 +3906,6 @@
           <t>SRT_DATE</t>
         </is>
       </c>
-      <c r="B92" t="inlineStr"/>
       <c r="C92" t="inlineStr">
         <is>
           <t>2026-08-15T06:44:18.832</t>
@@ -4095,7 +3923,6 @@
           <t>END_DATE</t>
         </is>
       </c>
-      <c r="B93" t="inlineStr"/>
       <c r="C93" t="inlineStr">
         <is>
           <t>2026-08-15T07:24:02.752</t>
@@ -4113,7 +3940,6 @@
           <t>FILETIME</t>
         </is>
       </c>
-      <c r="B94" t="inlineStr"/>
       <c r="C94" t="inlineStr">
         <is>
           <t>39.73200000000002</t>
@@ -4131,7 +3957,6 @@
           <t>VITLTIME</t>
         </is>
       </c>
-      <c r="B95" t="inlineStr"/>
       <c r="C95" t="inlineStr">
         <is>
           <t>38.638600185513496</t>
@@ -4149,7 +3974,6 @@
           <t>ONTARG</t>
         </is>
       </c>
-      <c r="B96" t="inlineStr"/>
       <c r="C96" t="inlineStr">
         <is>
           <t>100.0</t>
@@ -4167,7 +3991,6 @@
           <t>NKEEPOUT</t>
         </is>
       </c>
-      <c r="B97" t="inlineStr"/>
       <c r="C97" t="inlineStr">
         <is>
           <t>48.320413436692505</t>
@@ -4185,7 +4008,6 @@
           <t>VKEEPOUT</t>
         </is>
       </c>
-      <c r="B98" t="inlineStr"/>
       <c r="C98" t="inlineStr">
         <is>
           <t>21.44702842377261</t>
@@ -4203,7 +4025,6 @@
           <t>VITLMISS</t>
         </is>
       </c>
-      <c r="B99" t="inlineStr"/>
       <c r="C99" t="inlineStr">
         <is>
           <t>0.0</t>
@@ -4221,7 +4042,6 @@
           <t>TARGTIME</t>
         </is>
       </c>
-      <c r="B100" t="inlineStr"/>
       <c r="C100" t="inlineStr">
         <is>
           <t>False</t>
@@ -4239,7 +4059,6 @@
           <t>APCOMP1</t>
         </is>
       </c>
-      <c r="B101" t="inlineStr"/>
       <c r="C101" t="inlineStr">
         <is>
           <t>94.34050514499532</t>
@@ -4254,64 +4073,60 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>TARGCENT</t>
-        </is>
-      </c>
-      <c r="B102" t="inlineStr"/>
+          <t>TCENT10</t>
+        </is>
+      </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>0.92</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Target Centered</t>
+          <t>Fraction of time target within 10 px of center</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>TARGCOMP</t>
-        </is>
-      </c>
-      <c r="B103" t="inlineStr"/>
+          <t>TCENT20</t>
+        </is>
+      </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>0.97</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Target Complete</t>
+          <t>Fraction of time target within 20 px of center</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>DETTEMP1</t>
-        </is>
-      </c>
-      <c r="B104" t="inlineStr"/>
+          <t>TCENT30</t>
+        </is>
+      </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Cold Tip 1 temperature less than 140K</t>
+          <t>Fraction of time target within 30 px of center</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>DETTEMP2</t>
-        </is>
-      </c>
-      <c r="B105" t="inlineStr"/>
+          <t>TARGCOMP</t>
+        </is>
+      </c>
       <c r="C105" t="inlineStr">
         <is>
           <t>True</t>
@@ -4319,37 +4134,43 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Cold Tip 2 temperature less than 140K</t>
+          <t>Target Complete</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>COMMENT</t>
-        </is>
-      </c>
-      <c r="B106" t="inlineStr"/>
+          <t>DETTEMP1</t>
+        </is>
+      </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Appended WCS.</t>
-        </is>
-      </c>
-      <c r="D106" t="inlineStr"/>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Cold Tip 1 temperature less than 140K</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>COMMENT</t>
-        </is>
-      </c>
-      <c r="B107" t="inlineStr"/>
+          <t>DETTEMP2</t>
+        </is>
+      </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Appended Vectors.</t>
-        </is>
-      </c>
-      <c r="D107" t="inlineStr"/>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Cold Tip 2 temperature less than 140K</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -4357,13 +4178,35 @@
           <t>COMMENT</t>
         </is>
       </c>
-      <c r="B108" t="inlineStr"/>
       <c r="C108" t="inlineStr">
         <is>
           <t>Appended WCS.</t>
         </is>
       </c>
-      <c r="D108" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>COMMENT</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Appended Vectors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>COMMENT</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Appended WCS.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4473,13 +4316,11 @@
           <t>NAXIS1</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>80</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4487,13 +4328,11 @@
           <t>NAXIS2</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>250</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4501,13 +4340,11 @@
           <t>NAXIS3</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>387</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4515,7 +4352,6 @@
           <t>PCOUNT</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
           <t>0</t>
@@ -4533,7 +4369,6 @@
           <t>GCOUNT</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
           <t>1</t>
@@ -4573,7 +4408,6 @@
           <t>CHECKSUM</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
           <t>haAkkY7khaAkhY5k</t>
@@ -4591,7 +4425,6 @@
           <t>DATASUM</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
           <t>1725050178</t>
@@ -4609,13 +4442,11 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
           <t>ct / s</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4623,7 +4454,6 @@
           <t>WCSAXES</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
           <t>2</t>
@@ -4641,7 +4471,6 @@
           <t>CRPIX1</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
           <t>1781.0</t>
@@ -4659,7 +4488,6 @@
           <t>CRPIX2</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr">
         <is>
           <t>1085.0</t>
@@ -4677,7 +4505,6 @@
           <t>PC1_1</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr">
         <is>
           <t>0.92526147848475</t>
@@ -4695,7 +4522,6 @@
           <t>PC1_2</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
           <t>-0.37932993084148</t>
@@ -4713,7 +4539,6 @@
           <t>PC2_1</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
           <t>0.37932993084148</t>
@@ -4731,7 +4556,6 @@
           <t>PC2_2</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
           <t>0.92526147848475</t>
@@ -4749,7 +4573,6 @@
           <t>CDELT1</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
           <t>0.00033055555555556</t>
@@ -4767,7 +4590,6 @@
           <t>CDELT2</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
           <t>0.00033055555555556</t>
@@ -4785,7 +4607,6 @@
           <t>CUNIT1</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
           <t>deg</t>
@@ -4803,7 +4624,6 @@
           <t>CUNIT2</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
           <t>deg</t>
@@ -4821,7 +4641,6 @@
           <t>CTYPE1</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
           <t>RA---TAN</t>
@@ -4839,7 +4658,6 @@
           <t>CTYPE2</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
           <t>DEC--TAN</t>
@@ -4857,7 +4675,6 @@
           <t>CRVAL1</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
           <t>307.86216741569</t>
@@ -4875,7 +4692,6 @@
           <t>CRVAL2</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
           <t>39.938785328355</t>
@@ -4893,7 +4709,6 @@
           <t>LONPOLE</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
           <t>180.0</t>
@@ -4911,7 +4726,6 @@
           <t>LATPOLE</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
           <t>39.938785328355</t>
@@ -4929,7 +4743,6 @@
           <t>MJDREF</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
           <t>0.0</t>
@@ -4947,7 +4760,6 @@
           <t>RADESYS</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
           <t>ICRS</t>
@@ -4965,7 +4777,6 @@
           <t>WCSAXES</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
           <t>2</t>
@@ -4983,7 +4794,6 @@
           <t>CRPIX1</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
           <t>1781.0</t>
@@ -5001,7 +4811,6 @@
           <t>CRPIX2</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
           <t>1085.0</t>
@@ -5019,7 +4828,6 @@
           <t>PC1_1</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
           <t>0.92523789004974</t>
@@ -5037,7 +4845,6 @@
           <t>PC1_2</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
           <t>-0.3793874626504</t>
@@ -5055,7 +4862,6 @@
           <t>PC2_1</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
           <t>0.3793874626504</t>
@@ -5073,7 +4879,6 @@
           <t>PC2_2</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
           <t>0.92523789004974</t>
@@ -5091,7 +4896,6 @@
           <t>CDELT1</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
           <t>0.00033055555555556</t>
@@ -5109,7 +4913,6 @@
           <t>CDELT2</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
           <t>0.00033055555555556</t>
@@ -5127,7 +4930,6 @@
           <t>CUNIT1</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
           <t>deg</t>
@@ -5145,7 +4947,6 @@
           <t>CUNIT2</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
           <t>deg</t>
@@ -5163,7 +4964,6 @@
           <t>CTYPE1</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
           <t>RA---TAN</t>
@@ -5181,7 +4981,6 @@
           <t>CTYPE2</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
           <t>DEC--TAN</t>
@@ -5199,7 +4998,6 @@
           <t>CRVAL1</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
           <t>307.86215209961</t>
@@ -5217,7 +5015,6 @@
           <t>CRVAL2</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
           <t>39.938789367676</t>
@@ -5235,7 +5032,6 @@
           <t>LONPOLE</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr">
         <is>
           <t>180.0</t>
@@ -5253,7 +5049,6 @@
           <t>LATPOLE</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr">
         <is>
           <t>39.938789367676</t>
@@ -5271,7 +5066,6 @@
           <t>MJDREF</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr">
         <is>
           <t>0.0</t>
@@ -5289,7 +5083,6 @@
           <t>RADESYS</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr">
         <is>
           <t>ICRS</t>
@@ -5409,7 +5202,6 @@
           <t>NAXIS1</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>40</t>
@@ -5427,7 +5219,6 @@
           <t>NAXIS2</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>11718</t>
@@ -5445,7 +5236,6 @@
           <t>PCOUNT</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>0</t>
@@ -5463,7 +5253,6 @@
           <t>GCOUNT</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
           <t>1</t>
@@ -5513,7 +5302,6 @@
           <t>JD</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -5531,7 +5319,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -5549,7 +5336,6 @@
           <t>RightAscension</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -5567,7 +5353,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -5585,7 +5370,6 @@
           <t>Declination</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -5603,7 +5387,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -5621,7 +5404,6 @@
           <t>Rotation</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -5639,7 +5421,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -5657,7 +5438,6 @@
           <t>PCOTemp</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -5675,7 +5455,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -5693,7 +5472,6 @@
           <t>ASTROMETRY</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5701,7 +5479,6 @@
           <t>CHECKSUM</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
           <t>3UTa3SQY3SQa3SQY</t>
@@ -5719,7 +5496,6 @@
           <t>DATASUM</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
           <t>3190933090</t>
@@ -5839,13 +5615,11 @@
           <t>NAXIS1</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>387</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -5853,7 +5627,6 @@
           <t>PCOUNT</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>0</t>
@@ -5871,7 +5644,6 @@
           <t>GCOUNT</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>1</t>
@@ -5889,7 +5661,6 @@
           <t>FRAME</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
           <t>JD</t>
@@ -5929,7 +5700,6 @@
           <t>CHECKSUM</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
           <t>0He51Hc40Hc40Hc4</t>
@@ -5947,7 +5717,6 @@
           <t>DATASUM</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
           <t>4194533316</t>
@@ -6067,13 +5836,11 @@
           <t>NAXIS1</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>387</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -6081,7 +5848,6 @@
           <t>PCOUNT</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>0</t>
@@ -6099,7 +5865,6 @@
           <t>GCOUNT</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>1</t>
@@ -6117,7 +5882,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
           <t>second</t>
@@ -6157,7 +5921,6 @@
           <t>CHECKSUM</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
           <t>bKAlcI7kbIAkbI5k</t>
@@ -6175,7 +5938,6 @@
           <t>DATASUM</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
           <t>941144289</t>
@@ -6295,13 +6057,11 @@
           <t>NAXIS1</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>387</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -6309,7 +6069,6 @@
           <t>PCOUNT</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>0</t>
@@ -6327,7 +6086,6 @@
           <t>GCOUNT</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>1</t>
@@ -6367,7 +6125,6 @@
           <t>CHECKSUM</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
           <t>5XYF5VW95VWE5VW9</t>
@@ -6385,7 +6142,6 @@
           <t>DATASUM</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
           <t>74691</t>
@@ -6505,7 +6261,6 @@
           <t>NAXIS1</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>130</t>
@@ -6523,7 +6278,6 @@
           <t>NAXIS2</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>387</t>
@@ -6541,7 +6295,6 @@
           <t>PCOUNT</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>0</t>
@@ -6559,7 +6312,6 @@
           <t>GCOUNT</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
           <t>1</t>
@@ -6609,7 +6361,6 @@
           <t>avg_ra</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -6627,7 +6378,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -6645,7 +6395,6 @@
           <t>avg_dec</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -6663,7 +6412,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -6681,7 +6429,6 @@
           <t>avg_rot</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -6699,7 +6446,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -6717,7 +6463,6 @@
           <t>err_ra</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -6735,7 +6480,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -6753,7 +6497,6 @@
           <t>err_dec</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -6771,7 +6514,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -6789,7 +6531,6 @@
           <t>err_rot</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -6807,7 +6548,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -6825,7 +6565,6 @@
           <t>jd</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -6843,7 +6582,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -6861,7 +6599,6 @@
           <t>exptime</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -6879,7 +6616,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -6897,7 +6633,6 @@
           <t>target_sep</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -6915,7 +6650,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -6933,7 +6667,6 @@
           <t>vitl_frames_count</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -6951,7 +6684,6 @@
           <t>K</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -6969,7 +6701,6 @@
           <t>vitl_missing_frames</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -6987,7 +6718,6 @@
           <t>K</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -7005,7 +6735,6 @@
           <t>earth_angle</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -7023,7 +6752,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -7041,7 +6769,6 @@
           <t>earth_illumination</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -7059,7 +6786,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -7077,7 +6803,6 @@
           <t>sun_angle</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -7095,7 +6820,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -7113,7 +6837,6 @@
           <t>visda_keepout</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -7131,7 +6854,6 @@
           <t>L</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -7149,7 +6871,6 @@
           <t>nirda_keepout</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -7167,7 +6888,6 @@
           <t>L</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -7185,7 +6905,6 @@
           <t>posx</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -7203,7 +6922,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -7221,7 +6939,6 @@
           <t>posy</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -7239,7 +6956,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -7257,7 +6973,6 @@
           <t>VECTORS</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -7265,7 +6980,6 @@
           <t>CHECKSUM</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
           <t>nIJ7pHJ5nHJ5nHJ5</t>
@@ -7283,7 +6997,6 @@
           <t>DATASUM</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr">
         <is>
           <t>708805240</t>
@@ -7403,7 +7116,6 @@
           <t>NAXIS1</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>80</t>
@@ -7421,7 +7133,6 @@
           <t>NAXIS2</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>250</t>
@@ -7439,7 +7150,6 @@
           <t>PCOUNT</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>0</t>
@@ -7457,7 +7167,6 @@
           <t>GCOUNT</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
           <t>1</t>
@@ -7485,7 +7194,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -7503,7 +7211,6 @@
           <t>32768</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -7533,7 +7240,6 @@
           <t>CHECKSUM</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
           <t>95ajG4Ui94aiG4Ui</t>
@@ -7551,7 +7257,6 @@
           <t>DATASUM</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
           <t>335287306</t>

</xml_diff>

<commit_message>
Keep every NIRDA aperture row; exclude flagged pixels only
NIRDALevel1HDUList.aperture dropped every row (wavelength) that had
one QUALITY-flagged or contaminated pixel. Contamination bit 4 marks
any pixel with a trace of another star's light, so with correct NIR
scene fluxes this left 1 of 218 rows for HD 189733 and 6 of 218 for
TOI-181, and the inspection scores built on it (APCOMP1, TARGCOMP,
lc_med) collapsed.

The aperture is now the target pixels that are good in QUALITY.
Contaminated pixels are kept: in NIRDA they lie along dispersed
traces, and their light is a dilution reported by CONTAM. APCOMP1 is
now the percentage of target pixels usable in QUALITY.
</commit_message>
<xml_diff>
--- a/src/pandorafits/formats/nirda/level2_nirda.xlsx
+++ b/src/pandorafits/formats/nirda/level2_nirda.xlsx
@@ -1075,7 +1075,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1438,32 +1438,66 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CHECKSUM</t>
+          <t>MAGSRC</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>eD6kf93ieC3ie93i</t>
+          <t>j_m</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>HDU checksum updated 2026-09-09T15:46:12</t>
+          <t>Catalog magnitude used for scene fluxes</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>NOMAG</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Catalog stars without MAGSRC, given zero flux</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>CHECKSUM</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>eD6kf93ieC3ie93i</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>HDU checksum updated 2026-09-09T15:46:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>DATASUM</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>178391814</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>data unit checksum updated 2026-09-09T15:46:12</t>
         </is>

</xml_diff>

<commit_message>
Changes to soc report (#15)
* Changes TARGCENT to TCENT`n` which quantifies the fraction of a observation where data was within 10,20,30 pixels from center.

* Fixes issue where TARGCOMP was comparing percent to ratios

* Fixes issue where nan's were not being converted to the expected number
</commit_message>
<xml_diff>
--- a/src/pandorafits/formats/nirda/level2_nirda.xlsx
+++ b/src/pandorafits/formats/nirda/level2_nirda.xlsx
@@ -745,7 +745,6 @@
           <t>NAXIS1</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>32</t>
@@ -763,7 +762,6 @@
           <t>NAXIS2</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>250</t>
@@ -781,7 +779,6 @@
           <t>PCOUNT</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>0</t>
@@ -799,7 +796,6 @@
           <t>GCOUNT</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
           <t>1</t>
@@ -849,7 +845,6 @@
           <t>row</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -867,7 +862,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -875,13 +869,11 @@
           <t>TUNIT1</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
           <t>pix</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -899,7 +891,6 @@
           <t>drow</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -917,7 +908,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -925,13 +915,11 @@
           <t>TUNIT2</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
           <t>pix</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -949,7 +937,6 @@
           <t>wavelength</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -967,7 +954,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -975,13 +961,11 @@
           <t>TUNIT3</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
           <t>um</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -999,7 +983,6 @@
           <t>sensitivity</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1017,7 +1000,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1025,13 +1007,11 @@
           <t>TUNIT4</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
           <t>cm2 Angstrom count erg-1</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1049,7 +1029,6 @@
           <t>WAVELENGTH_SOLUTION</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1057,7 +1036,6 @@
           <t>CHECKSUM</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
           <t>9M5MFM5K9M5KEM5K</t>
@@ -1075,7 +1053,6 @@
           <t>DATASUM</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
           <t>2322579671</t>
@@ -1195,7 +1172,6 @@
           <t>NAXIS1</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>80</t>
@@ -1213,7 +1189,6 @@
           <t>NAXIS2</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>250</t>
@@ -1231,7 +1206,6 @@
           <t>PCOUNT</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>0</t>
@@ -1249,7 +1223,6 @@
           <t>GCOUNT</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
           <t>1</t>
@@ -1289,7 +1262,6 @@
           <t>CONTAM</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
           <t>1.45948781805724e-05</t>
@@ -1307,7 +1279,6 @@
           <t>COMPLTE</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
           <t>1.0001196545262074</t>
@@ -1325,7 +1296,6 @@
           <t>TOTAP</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
           <t>6054546.661906874</t>
@@ -1343,13 +1313,11 @@
           <t>RA</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
           <t>307.85996711980397</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1357,13 +1325,11 @@
           <t>DEC</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
           <t>39.93898084328189</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1371,13 +1337,11 @@
           <t>ROW</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
           <t>1086.4587761921186</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1385,13 +1349,11 @@
           <t>COLUMN</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr">
         <is>
           <t>1775.530593149113</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1399,13 +1361,11 @@
           <t>GAIA_ID</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr">
         <is>
           <t>2064327278651198336</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1413,7 +1373,6 @@
           <t>IMSIZE0</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
           <t>250</t>
@@ -1431,7 +1390,6 @@
           <t>IMCRNR0</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
           <t>962</t>
@@ -1449,7 +1407,6 @@
           <t>IMSIZE1</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
           <t>80</t>
@@ -1467,7 +1424,6 @@
           <t>IMCRNR1</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
           <t>1737</t>
@@ -1485,7 +1441,6 @@
           <t>CHECKSUM</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
           <t>eD6kf93ieC3ie93i</t>
@@ -1503,7 +1458,6 @@
           <t>DATASUM</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
           <t>178391814</t>
@@ -1623,7 +1577,6 @@
           <t>NAXIS1</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>80</t>
@@ -1641,7 +1594,6 @@
           <t>NAXIS2</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>250</t>
@@ -1659,7 +1611,6 @@
           <t>PCOUNT</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>0</t>
@@ -1677,7 +1628,6 @@
           <t>GCOUNT</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
           <t>1</t>
@@ -1695,7 +1645,6 @@
           <t>WCSAXES</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
           <t>2</t>
@@ -1713,7 +1662,6 @@
           <t>CRPIX1</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
           <t>44.0</t>
@@ -1731,7 +1679,6 @@
           <t>CRPIX2</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
           <t>123.0</t>
@@ -1749,7 +1696,6 @@
           <t>PC1_1</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
           <t>0.92523789004974</t>
@@ -1767,7 +1713,6 @@
           <t>PC1_2</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
           <t>-0.3793874626504</t>
@@ -1785,7 +1730,6 @@
           <t>PC2_1</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
           <t>0.3793874626504</t>
@@ -1803,7 +1747,6 @@
           <t>PC2_2</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
           <t>0.92523789004974</t>
@@ -1821,7 +1764,6 @@
           <t>CDELT1</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr">
         <is>
           <t>0.00033055555555556</t>
@@ -1839,7 +1781,6 @@
           <t>CDELT2</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr">
         <is>
           <t>0.00033055555555556</t>
@@ -1857,7 +1798,6 @@
           <t>CUNIT1</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
           <t>deg</t>
@@ -1875,7 +1815,6 @@
           <t>CUNIT2</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
           <t>deg</t>
@@ -1893,7 +1832,6 @@
           <t>CTYPE1</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
           <t>RA---TAN</t>
@@ -1911,7 +1849,6 @@
           <t>CTYPE2</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
           <t>DEC--TAN</t>
@@ -1929,7 +1866,6 @@
           <t>CRVAL1</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
           <t>307.86215209961</t>
@@ -1947,7 +1883,6 @@
           <t>CRVAL2</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
           <t>39.938789367676</t>
@@ -1965,7 +1900,6 @@
           <t>LONPOLE</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
           <t>180.0</t>
@@ -1983,7 +1917,6 @@
           <t>LATPOLE</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
           <t>39.938789367676</t>
@@ -2001,7 +1934,6 @@
           <t>MJDREF</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
           <t>0.0</t>
@@ -2019,7 +1951,6 @@
           <t>RADESYS</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
           <t>ICRS</t>
@@ -2059,7 +1990,6 @@
           <t>IMSIZE0</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
           <t>250</t>
@@ -2077,7 +2007,6 @@
           <t>IMCRNR0</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
           <t>962</t>
@@ -2095,7 +2024,6 @@
           <t>IMSIZE1</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
           <t>80</t>
@@ -2113,7 +2041,6 @@
           <t>IMCRNR1</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
           <t>1737</t>
@@ -2131,7 +2058,6 @@
           <t>CHECKSUM</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
           <t>LF7VOD4VLD4VLD4V</t>
@@ -2149,7 +2075,6 @@
           <t>DATASUM</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
           <t>4243662291</t>
@@ -2269,7 +2194,6 @@
           <t>NAXIS1</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>250</t>
@@ -2287,7 +2211,6 @@
           <t>NAXIS2</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>387</t>
@@ -2305,7 +2228,6 @@
           <t>PCOUNT</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>0</t>
@@ -2323,7 +2245,6 @@
           <t>GCOUNT</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
           <t>1</t>
@@ -2341,13 +2262,11 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
           <t>ct / s</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2377,7 +2296,6 @@
           <t>CHECKSUM</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
           <t>a0AUc06Ta0ATa03T</t>
@@ -2395,7 +2313,6 @@
           <t>DATASUM</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
           <t>4262218308</t>
@@ -2418,7 +2335,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D108"/>
+  <dimension ref="A1:D110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2525,7 +2442,6 @@
           <t>True</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2555,7 +2471,6 @@
           <t>NEXTEND</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>2</t>
@@ -2573,7 +2488,6 @@
           <t>SIMDATA</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
           <t>False</t>
@@ -2591,7 +2505,6 @@
           <t>SCIDATA</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
           <t>True</t>
@@ -2675,7 +2588,6 @@
           <t>CREATOR</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
           <t>Pandora MOC</t>
@@ -2693,7 +2605,6 @@
           <t>CRSOFTV</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
           <t>v3.06</t>
@@ -2711,7 +2622,6 @@
           <t>COMPTYPE</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
           <t>1</t>
@@ -2729,7 +2639,6 @@
           <t>TRANSID</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr">
         <is>
           <t>0</t>
@@ -2747,7 +2656,6 @@
           <t>TARG_ID</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr">
         <is>
           <t>KELT-9b</t>
@@ -2765,7 +2673,6 @@
           <t>FILENAME</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
           <t>/sssp/data/2026/08/15/2026-08-15__06-44-18_InfImg_KELT-9b_d0080x0250x3096_b1_e01_i387_g02_d16_r04.sp</t>
@@ -2783,7 +2690,6 @@
           <t>BINSIZE</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
           <t>1</t>
@@ -2801,7 +2707,6 @@
           <t>BITDEPTH</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
           <t>32</t>
@@ -2819,7 +2724,6 @@
           <t>BITSPIX</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
           <t>16</t>
@@ -2837,7 +2741,6 @@
           <t>ROISTRTX</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
           <t>1737</t>
@@ -2855,7 +2758,6 @@
           <t>ROISTRTY</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
           <t>962</t>
@@ -2873,7 +2775,6 @@
           <t>ROISTRTZ</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
           <t>0</t>
@@ -2891,7 +2792,6 @@
           <t>ROISIZEX</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
           <t>80</t>
@@ -2909,7 +2809,6 @@
           <t>ROISIZEY</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
           <t>250</t>
@@ -2927,7 +2826,6 @@
           <t>ROISIZEZ</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
           <t>774</t>
@@ -2945,7 +2843,6 @@
           <t>RICEX</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
           <t>5</t>
@@ -2963,7 +2860,6 @@
           <t>RICEY</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
           <t>28</t>
@@ -2981,7 +2877,6 @@
           <t>CORSTIME</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
           <t>840091495</t>
@@ -2999,7 +2894,6 @@
           <t>FINETIME</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
           <t>832000000</t>
@@ -3017,7 +2911,6 @@
           <t>COMMAND</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
           <t>10</t>
@@ -3035,7 +2928,6 @@
           <t>CONFIG1</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
           <t>53251</t>
@@ -3053,7 +2945,6 @@
           <t>CONFIG2</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
           <t>0</t>
@@ -3071,7 +2962,6 @@
           <t>CONFIG3</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
           <t>0</t>
@@ -3089,7 +2979,6 @@
           <t>GAINREG</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
           <t>37002</t>
@@ -3107,7 +2996,6 @@
           <t>RESETS1</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
           <t>259</t>
@@ -3125,7 +3013,6 @@
           <t>RESETS2</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
           <t>1</t>
@@ -3143,7 +3030,6 @@
           <t>DROPS1</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
           <t>1</t>
@@ -3161,7 +3047,6 @@
           <t>DROPS2</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
           <t>16</t>
@@ -3179,7 +3064,6 @@
           <t>DROPS3</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
           <t>0</t>
@@ -3197,7 +3081,6 @@
           <t>READS</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
           <t>4</t>
@@ -3215,7 +3098,6 @@
           <t>GRPS</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
           <t>2</t>
@@ -3233,7 +3115,6 @@
           <t>INTEGRTS</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
           <t>387</t>
@@ -3251,7 +3132,6 @@
           <t>EXPOSRES</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
           <t>1</t>
@@ -3269,7 +3149,6 @@
           <t>ENDDELAY</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
           <t>0</t>
@@ -3287,7 +3166,6 @@
           <t>RSTSINC</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
           <t>0</t>
@@ -3305,7 +3183,6 @@
           <t>DRPSINC</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr">
         <is>
           <t>0</t>
@@ -3323,7 +3200,6 @@
           <t>FRMSTOT</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr">
         <is>
           <t>10320</t>
@@ -3341,7 +3217,6 @@
           <t>FRMSEXP</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr">
         <is>
           <t>3096</t>
@@ -3359,7 +3234,6 @@
           <t>FRMSACQ</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr">
         <is>
           <t>3096</t>
@@ -3377,7 +3251,6 @@
           <t>GRPSAVGD</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr">
         <is>
           <t>1</t>
@@ -3395,7 +3268,6 @@
           <t>PAMPGAIN</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr">
         <is>
           <t>5.65685</t>
@@ -3413,7 +3285,6 @@
           <t>FRMTIME</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr">
         <is>
           <t>231</t>
@@ -3431,7 +3302,6 @@
           <t>TSIDECAR</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr">
         <is>
           <t>3.3816466331481934</t>
@@ -3449,7 +3319,6 @@
           <t>TCOMPRJT</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr">
         <is>
           <t>278.990966796875</t>
@@ -3467,7 +3336,6 @@
           <t>TCLDTIP1</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr"/>
       <c r="C57" t="inlineStr">
         <is>
           <t>131.50372314453125</t>
@@ -3485,7 +3353,6 @@
           <t>TCLDTIP2</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr"/>
       <c r="C58" t="inlineStr">
         <is>
           <t>120.03438568115234</t>
@@ -3503,7 +3370,6 @@
           <t>CHECKSUM</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr">
         <is>
           <t>9agDGWgC9agCEWgC</t>
@@ -3521,7 +3387,6 @@
           <t>DATASUM</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr">
         <is>
           <t>0</t>
@@ -3539,13 +3404,11 @@
           <t>FIXED</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr"/>
       <c r="C61" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3553,13 +3416,11 @@
           <t>PFSOFTV</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr"/>
       <c r="C62" t="inlineStr">
         <is>
           <t>0.6.0</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3567,13 +3428,11 @@
           <t>PRSOFTV</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr"/>
       <c r="C63" t="inlineStr">
         <is>
           <t>2.9.1</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3581,13 +3440,11 @@
           <t>PFCLASS</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr"/>
       <c r="C64" t="inlineStr">
         <is>
           <t>NIRDALevel2HDUList</t>
         </is>
       </c>
-      <c r="D64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3595,7 +3452,6 @@
           <t>PFTIME</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr"/>
       <c r="C65" t="inlineStr">
         <is>
           <t>2026-09-09T19:46:08.484</t>
@@ -3613,7 +3469,6 @@
           <t>TARG_RA</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr"/>
       <c r="C66" t="inlineStr">
         <is>
           <t>307.8599548339844</t>
@@ -3631,7 +3486,6 @@
           <t>TARG_DEC</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr"/>
       <c r="C67" t="inlineStr">
         <is>
           <t>39.9389762878418</t>
@@ -3649,7 +3503,6 @@
           <t>RA</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr"/>
       <c r="C68" t="inlineStr">
         <is>
           <t>307.86216741569376</t>
@@ -3667,7 +3520,6 @@
           <t>DEC</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr"/>
       <c r="C69" t="inlineStr">
         <is>
           <t>39.93878532835476</t>
@@ -3685,7 +3537,6 @@
           <t>ROLL</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr"/>
       <c r="C70" t="inlineStr">
         <is>
           <t>247.7078167885557</t>
@@ -3703,7 +3554,6 @@
           <t>POSX</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr"/>
       <c r="C71" t="inlineStr">
         <is>
           <t>1775.498998065344</t>
@@ -3721,7 +3571,6 @@
           <t>POSY</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr"/>
       <c r="C72" t="inlineStr">
         <is>
           <t>1086.4568375724239</t>
@@ -3739,7 +3588,6 @@
           <t>GAIADR3</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr"/>
       <c r="C73" t="inlineStr">
         <is>
           <t>Gaia DR3 2064327278651198336</t>
@@ -3757,7 +3605,6 @@
           <t>GAIARA</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr"/>
       <c r="C74" t="inlineStr">
         <is>
           <t>307.8599027970418</t>
@@ -3775,7 +3622,6 @@
           <t>GAIADEC</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr"/>
       <c r="C75" t="inlineStr">
         <is>
           <t>39.93891900336815</t>
@@ -3793,7 +3639,6 @@
           <t>PARALLAX</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr"/>
       <c r="C76" t="inlineStr">
         <is>
           <t>4.825836101438949</t>
@@ -3811,7 +3656,6 @@
           <t>PMRA</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr"/>
       <c r="C77" t="inlineStr">
         <is>
           <t>16.716578051403854</t>
@@ -3829,7 +3673,6 @@
           <t>PMDEC</t>
         </is>
       </c>
-      <c r="B78" t="inlineStr"/>
       <c r="C78" t="inlineStr">
         <is>
           <t>20.96090596020299</t>
@@ -3847,7 +3690,6 @@
           <t>2MASSID</t>
         </is>
       </c>
-      <c r="B79" t="inlineStr"/>
       <c r="C79" t="inlineStr">
         <is>
           <t>2MASS J20312634+3956196</t>
@@ -3865,7 +3707,6 @@
           <t>J_M</t>
         </is>
       </c>
-      <c r="B80" t="inlineStr"/>
       <c r="C80" t="inlineStr">
         <is>
           <t>7.458</t>
@@ -3883,7 +3724,6 @@
           <t>H_M</t>
         </is>
       </c>
-      <c r="B81" t="inlineStr"/>
       <c r="C81" t="inlineStr">
         <is>
           <t>7.492</t>
@@ -3901,7 +3741,6 @@
           <t>K_M</t>
         </is>
       </c>
-      <c r="B82" t="inlineStr"/>
       <c r="C82" t="inlineStr">
         <is>
           <t>7.482</t>
@@ -3919,7 +3758,6 @@
           <t>G_M</t>
         </is>
       </c>
-      <c r="B83" t="inlineStr"/>
       <c r="C83" t="inlineStr">
         <is>
           <t>7.5902658552584015</t>
@@ -3937,7 +3775,6 @@
           <t>BP_M</t>
         </is>
       </c>
-      <c r="B84" t="inlineStr"/>
       <c r="C84" t="inlineStr">
         <is>
           <t>7.594925828938212</t>
@@ -3955,7 +3792,6 @@
           <t>RP_M</t>
         </is>
       </c>
-      <c r="B85" t="inlineStr"/>
       <c r="C85" t="inlineStr">
         <is>
           <t>7.552309075270038</t>
@@ -3973,7 +3809,6 @@
           <t>TEFF</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr"/>
       <c r="C86" t="inlineStr">
         <is>
           <t>9951.392</t>
@@ -3991,7 +3826,6 @@
           <t>LOGG</t>
         </is>
       </c>
-      <c r="B87" t="inlineStr"/>
       <c r="C87" t="inlineStr">
         <is>
           <t>3.9497</t>
@@ -4009,13 +3843,11 @@
           <t>COLLAPS</t>
         </is>
       </c>
-      <c r="B88" t="inlineStr"/>
       <c r="C88" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -4023,7 +3855,6 @@
           <t>BKG10</t>
         </is>
       </c>
-      <c r="B89" t="inlineStr"/>
       <c r="C89" t="inlineStr">
         <is>
           <t>119.15584415584416</t>
@@ -4041,7 +3872,6 @@
           <t>BKG50</t>
         </is>
       </c>
-      <c r="B90" t="inlineStr"/>
       <c r="C90" t="inlineStr">
         <is>
           <t>157.034632034632</t>
@@ -4059,7 +3889,6 @@
           <t>BKG90</t>
         </is>
       </c>
-      <c r="B91" t="inlineStr"/>
       <c r="C91" t="inlineStr">
         <is>
           <t>188.3116883116883</t>
@@ -4077,7 +3906,6 @@
           <t>SRT_DATE</t>
         </is>
       </c>
-      <c r="B92" t="inlineStr"/>
       <c r="C92" t="inlineStr">
         <is>
           <t>2026-08-15T06:44:18.832</t>
@@ -4095,7 +3923,6 @@
           <t>END_DATE</t>
         </is>
       </c>
-      <c r="B93" t="inlineStr"/>
       <c r="C93" t="inlineStr">
         <is>
           <t>2026-08-15T07:24:02.752</t>
@@ -4113,7 +3940,6 @@
           <t>FILETIME</t>
         </is>
       </c>
-      <c r="B94" t="inlineStr"/>
       <c r="C94" t="inlineStr">
         <is>
           <t>39.73200000000002</t>
@@ -4131,7 +3957,6 @@
           <t>VITLTIME</t>
         </is>
       </c>
-      <c r="B95" t="inlineStr"/>
       <c r="C95" t="inlineStr">
         <is>
           <t>38.638600185513496</t>
@@ -4149,7 +3974,6 @@
           <t>ONTARG</t>
         </is>
       </c>
-      <c r="B96" t="inlineStr"/>
       <c r="C96" t="inlineStr">
         <is>
           <t>100.0</t>
@@ -4167,7 +3991,6 @@
           <t>NKEEPOUT</t>
         </is>
       </c>
-      <c r="B97" t="inlineStr"/>
       <c r="C97" t="inlineStr">
         <is>
           <t>48.320413436692505</t>
@@ -4185,7 +4008,6 @@
           <t>VKEEPOUT</t>
         </is>
       </c>
-      <c r="B98" t="inlineStr"/>
       <c r="C98" t="inlineStr">
         <is>
           <t>21.44702842377261</t>
@@ -4203,7 +4025,6 @@
           <t>VITLMISS</t>
         </is>
       </c>
-      <c r="B99" t="inlineStr"/>
       <c r="C99" t="inlineStr">
         <is>
           <t>0.0</t>
@@ -4221,7 +4042,6 @@
           <t>TARGTIME</t>
         </is>
       </c>
-      <c r="B100" t="inlineStr"/>
       <c r="C100" t="inlineStr">
         <is>
           <t>False</t>
@@ -4239,7 +4059,6 @@
           <t>APCOMP1</t>
         </is>
       </c>
-      <c r="B101" t="inlineStr"/>
       <c r="C101" t="inlineStr">
         <is>
           <t>94.34050514499532</t>
@@ -4254,64 +4073,60 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>TARGCENT</t>
-        </is>
-      </c>
-      <c r="B102" t="inlineStr"/>
+          <t>TCENT10</t>
+        </is>
+      </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>0.92</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Target Centered</t>
+          <t>Fraction of time target within 10 px of center</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>TARGCOMP</t>
-        </is>
-      </c>
-      <c r="B103" t="inlineStr"/>
+          <t>TCENT20</t>
+        </is>
+      </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>0.97</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Target Complete</t>
+          <t>Fraction of time target within 20 px of center</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>DETTEMP1</t>
-        </is>
-      </c>
-      <c r="B104" t="inlineStr"/>
+          <t>TCENT30</t>
+        </is>
+      </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Cold Tip 1 temperature less than 140K</t>
+          <t>Fraction of time target within 30 px of center</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>DETTEMP2</t>
-        </is>
-      </c>
-      <c r="B105" t="inlineStr"/>
+          <t>TARGCOMP</t>
+        </is>
+      </c>
       <c r="C105" t="inlineStr">
         <is>
           <t>True</t>
@@ -4319,37 +4134,43 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Cold Tip 2 temperature less than 140K</t>
+          <t>Over 70% of target aperture pixels usable</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>COMMENT</t>
-        </is>
-      </c>
-      <c r="B106" t="inlineStr"/>
+          <t>DETTEMP1</t>
+        </is>
+      </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Appended WCS.</t>
-        </is>
-      </c>
-      <c r="D106" t="inlineStr"/>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Cold Tip 1 temperature less than 140K</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>COMMENT</t>
-        </is>
-      </c>
-      <c r="B107" t="inlineStr"/>
+          <t>DETTEMP2</t>
+        </is>
+      </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Appended Vectors.</t>
-        </is>
-      </c>
-      <c r="D107" t="inlineStr"/>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Cold Tip 2 temperature less than 140K</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -4357,13 +4178,35 @@
           <t>COMMENT</t>
         </is>
       </c>
-      <c r="B108" t="inlineStr"/>
       <c r="C108" t="inlineStr">
         <is>
           <t>Appended WCS.</t>
         </is>
       </c>
-      <c r="D108" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>COMMENT</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Appended Vectors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>COMMENT</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Appended WCS.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4473,13 +4316,11 @@
           <t>NAXIS1</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>80</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4487,13 +4328,11 @@
           <t>NAXIS2</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>250</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4501,13 +4340,11 @@
           <t>NAXIS3</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>387</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4515,7 +4352,6 @@
           <t>PCOUNT</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
           <t>0</t>
@@ -4533,7 +4369,6 @@
           <t>GCOUNT</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
           <t>1</t>
@@ -4573,7 +4408,6 @@
           <t>CHECKSUM</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
           <t>haAkkY7khaAkhY5k</t>
@@ -4591,7 +4425,6 @@
           <t>DATASUM</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
           <t>1725050178</t>
@@ -4609,13 +4442,11 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
           <t>ct / s</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4623,7 +4454,6 @@
           <t>WCSAXES</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
           <t>2</t>
@@ -4641,7 +4471,6 @@
           <t>CRPIX1</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
           <t>1781.0</t>
@@ -4659,7 +4488,6 @@
           <t>CRPIX2</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr">
         <is>
           <t>1085.0</t>
@@ -4677,7 +4505,6 @@
           <t>PC1_1</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr">
         <is>
           <t>0.92526147848475</t>
@@ -4695,7 +4522,6 @@
           <t>PC1_2</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
           <t>-0.37932993084148</t>
@@ -4713,7 +4539,6 @@
           <t>PC2_1</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
           <t>0.37932993084148</t>
@@ -4731,7 +4556,6 @@
           <t>PC2_2</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
           <t>0.92526147848475</t>
@@ -4749,7 +4573,6 @@
           <t>CDELT1</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
           <t>0.00033055555555556</t>
@@ -4767,7 +4590,6 @@
           <t>CDELT2</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
           <t>0.00033055555555556</t>
@@ -4785,7 +4607,6 @@
           <t>CUNIT1</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
           <t>deg</t>
@@ -4803,7 +4624,6 @@
           <t>CUNIT2</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
           <t>deg</t>
@@ -4821,7 +4641,6 @@
           <t>CTYPE1</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
           <t>RA---TAN</t>
@@ -4839,7 +4658,6 @@
           <t>CTYPE2</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
           <t>DEC--TAN</t>
@@ -4857,7 +4675,6 @@
           <t>CRVAL1</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
           <t>307.86216741569</t>
@@ -4875,7 +4692,6 @@
           <t>CRVAL2</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
           <t>39.938785328355</t>
@@ -4893,7 +4709,6 @@
           <t>LONPOLE</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
           <t>180.0</t>
@@ -4911,7 +4726,6 @@
           <t>LATPOLE</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
           <t>39.938785328355</t>
@@ -4929,7 +4743,6 @@
           <t>MJDREF</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
           <t>0.0</t>
@@ -4947,7 +4760,6 @@
           <t>RADESYS</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
           <t>ICRS</t>
@@ -4965,7 +4777,6 @@
           <t>WCSAXES</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
           <t>2</t>
@@ -4983,7 +4794,6 @@
           <t>CRPIX1</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
           <t>1781.0</t>
@@ -5001,7 +4811,6 @@
           <t>CRPIX2</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
           <t>1085.0</t>
@@ -5019,7 +4828,6 @@
           <t>PC1_1</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
           <t>0.92523789004974</t>
@@ -5037,7 +4845,6 @@
           <t>PC1_2</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
           <t>-0.3793874626504</t>
@@ -5055,7 +4862,6 @@
           <t>PC2_1</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
           <t>0.3793874626504</t>
@@ -5073,7 +4879,6 @@
           <t>PC2_2</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
           <t>0.92523789004974</t>
@@ -5091,7 +4896,6 @@
           <t>CDELT1</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
           <t>0.00033055555555556</t>
@@ -5109,7 +4913,6 @@
           <t>CDELT2</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
           <t>0.00033055555555556</t>
@@ -5127,7 +4930,6 @@
           <t>CUNIT1</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
           <t>deg</t>
@@ -5145,7 +4947,6 @@
           <t>CUNIT2</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
           <t>deg</t>
@@ -5163,7 +4964,6 @@
           <t>CTYPE1</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
           <t>RA---TAN</t>
@@ -5181,7 +4981,6 @@
           <t>CTYPE2</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
           <t>DEC--TAN</t>
@@ -5199,7 +4998,6 @@
           <t>CRVAL1</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
           <t>307.86215209961</t>
@@ -5217,7 +5015,6 @@
           <t>CRVAL2</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
           <t>39.938789367676</t>
@@ -5235,7 +5032,6 @@
           <t>LONPOLE</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr">
         <is>
           <t>180.0</t>
@@ -5253,7 +5049,6 @@
           <t>LATPOLE</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr">
         <is>
           <t>39.938789367676</t>
@@ -5271,7 +5066,6 @@
           <t>MJDREF</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr">
         <is>
           <t>0.0</t>
@@ -5289,7 +5083,6 @@
           <t>RADESYS</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr">
         <is>
           <t>ICRS</t>
@@ -5409,7 +5202,6 @@
           <t>NAXIS1</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>40</t>
@@ -5427,7 +5219,6 @@
           <t>NAXIS2</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>11718</t>
@@ -5445,7 +5236,6 @@
           <t>PCOUNT</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>0</t>
@@ -5463,7 +5253,6 @@
           <t>GCOUNT</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
           <t>1</t>
@@ -5513,7 +5302,6 @@
           <t>JD</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -5531,7 +5319,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -5549,7 +5336,6 @@
           <t>RightAscension</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -5567,7 +5353,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -5585,7 +5370,6 @@
           <t>Declination</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -5603,7 +5387,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -5621,7 +5404,6 @@
           <t>Rotation</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -5639,7 +5421,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -5657,7 +5438,6 @@
           <t>PCOTemp</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -5675,7 +5455,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -5693,7 +5472,6 @@
           <t>ASTROMETRY</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5701,7 +5479,6 @@
           <t>CHECKSUM</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
           <t>3UTa3SQY3SQa3SQY</t>
@@ -5719,7 +5496,6 @@
           <t>DATASUM</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
           <t>3190933090</t>
@@ -5839,13 +5615,11 @@
           <t>NAXIS1</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>387</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -5853,7 +5627,6 @@
           <t>PCOUNT</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>0</t>
@@ -5871,7 +5644,6 @@
           <t>GCOUNT</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>1</t>
@@ -5889,7 +5661,6 @@
           <t>FRAME</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
           <t>JD</t>
@@ -5929,7 +5700,6 @@
           <t>CHECKSUM</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
           <t>0He51Hc40Hc40Hc4</t>
@@ -5947,7 +5717,6 @@
           <t>DATASUM</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
           <t>4194533316</t>
@@ -6067,13 +5836,11 @@
           <t>NAXIS1</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>387</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -6081,7 +5848,6 @@
           <t>PCOUNT</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>0</t>
@@ -6099,7 +5865,6 @@
           <t>GCOUNT</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>1</t>
@@ -6117,7 +5882,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
           <t>second</t>
@@ -6157,7 +5921,6 @@
           <t>CHECKSUM</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
           <t>bKAlcI7kbIAkbI5k</t>
@@ -6175,7 +5938,6 @@
           <t>DATASUM</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
           <t>941144289</t>
@@ -6295,13 +6057,11 @@
           <t>NAXIS1</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>387</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -6309,7 +6069,6 @@
           <t>PCOUNT</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>0</t>
@@ -6327,7 +6086,6 @@
           <t>GCOUNT</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>1</t>
@@ -6367,7 +6125,6 @@
           <t>CHECKSUM</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
           <t>5XYF5VW95VWE5VW9</t>
@@ -6385,7 +6142,6 @@
           <t>DATASUM</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
           <t>74691</t>
@@ -6505,7 +6261,6 @@
           <t>NAXIS1</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>130</t>
@@ -6523,7 +6278,6 @@
           <t>NAXIS2</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>387</t>
@@ -6541,7 +6295,6 @@
           <t>PCOUNT</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>0</t>
@@ -6559,7 +6312,6 @@
           <t>GCOUNT</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
           <t>1</t>
@@ -6609,7 +6361,6 @@
           <t>avg_ra</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -6627,7 +6378,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -6645,7 +6395,6 @@
           <t>avg_dec</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -6663,7 +6412,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -6681,7 +6429,6 @@
           <t>avg_rot</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -6699,7 +6446,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -6717,7 +6463,6 @@
           <t>err_ra</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -6735,7 +6480,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -6753,7 +6497,6 @@
           <t>err_dec</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -6771,7 +6514,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -6789,7 +6531,6 @@
           <t>err_rot</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -6807,7 +6548,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -6825,7 +6565,6 @@
           <t>jd</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -6843,7 +6582,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -6861,7 +6599,6 @@
           <t>exptime</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -6879,7 +6616,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -6897,7 +6633,6 @@
           <t>target_sep</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -6915,7 +6650,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -6933,7 +6667,6 @@
           <t>vitl_frames_count</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -6951,7 +6684,6 @@
           <t>K</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -6969,7 +6701,6 @@
           <t>vitl_missing_frames</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -6987,7 +6718,6 @@
           <t>K</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -7005,7 +6735,6 @@
           <t>earth_angle</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -7023,7 +6752,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -7041,7 +6769,6 @@
           <t>earth_illumination</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -7059,7 +6786,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -7077,7 +6803,6 @@
           <t>sun_angle</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -7095,7 +6820,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -7113,7 +6837,6 @@
           <t>visda_keepout</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -7131,7 +6854,6 @@
           <t>L</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -7149,7 +6871,6 @@
           <t>nirda_keepout</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -7167,7 +6888,6 @@
           <t>L</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -7185,7 +6905,6 @@
           <t>posx</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -7203,7 +6922,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -7221,7 +6939,6 @@
           <t>posy</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -7239,7 +6956,6 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -7257,7 +6973,6 @@
           <t>VECTORS</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -7265,7 +6980,6 @@
           <t>CHECKSUM</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
           <t>nIJ7pHJ5nHJ5nHJ5</t>
@@ -7283,7 +6997,6 @@
           <t>DATASUM</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr">
         <is>
           <t>708805240</t>
@@ -7403,7 +7116,6 @@
           <t>NAXIS1</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>80</t>
@@ -7421,7 +7133,6 @@
           <t>NAXIS2</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>250</t>
@@ -7439,7 +7150,6 @@
           <t>PCOUNT</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>0</t>
@@ -7457,7 +7167,6 @@
           <t>GCOUNT</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
           <t>1</t>
@@ -7485,7 +7194,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -7503,7 +7211,6 @@
           <t>32768</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -7533,7 +7240,6 @@
           <t>CHECKSUM</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
           <t>95ajG4Ui94aiG4Ui</t>
@@ -7551,7 +7257,6 @@
           <t>DATASUM</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
           <t>335287306</t>

</xml_diff>